<commit_message>
Update BOM for Hyperboard 2
</commit_message>
<xml_diff>
--- a/notes/Hyperboard-Rev-2/AVIELF2HYPERBOARD-BOM.xlsx
+++ b/notes/Hyperboard-Rev-2/AVIELF2HYPERBOARD-BOM.xlsx
@@ -5,12 +5,12 @@
   <workbookPr dateCompatibility="0" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andrewwasson/Development/avi-elf-ii/notes/Hyperboard/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andrewwasson/Development/avi-elf-ii/notes/Hyperboard-Rev-2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{62C951AE-3A03-8043-8A47-AFA3795FF986}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{22AE9F18-3956-294F-B4CF-C23D6ACB0B78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22360" yWindow="8220" windowWidth="37800" windowHeight="20080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2980" yWindow="4180" windowWidth="37800" windowHeight="20080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Digikey.ca" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="304" uniqueCount="172">
+<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="328" uniqueCount="183">
   <si>
     <t>A1, A2</t>
   </si>
@@ -541,7 +541,40 @@
     <t>https://www.digikey.com/en/products/detail/adam-tech/PH2-80-UA/9830504</t>
   </si>
   <si>
-    <t>D9, D10, D11, D12, D13, D14, D15, D16, D17, D18, D19, D20, D21</t>
+    <t>U1</t>
+  </si>
+  <si>
+    <t>CD74HC151E</t>
+  </si>
+  <si>
+    <t>IC MULTIPLEXER 1 X 8:1 16-PDIP</t>
+  </si>
+  <si>
+    <t>https://www.digikey.ca/en/products/detail/texas-instruments/CD74HC151E/1506669</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/texas-instruments/CD74HC151E/1506669</t>
+  </si>
+  <si>
+    <t>RN3</t>
+  </si>
+  <si>
+    <t>RES ARRAY 8 RES 22K OHM 9SIP</t>
+  </si>
+  <si>
+    <t>SW1</t>
+  </si>
+  <si>
+    <t>Dip Switch SPST 8 Position</t>
+  </si>
+  <si>
+    <t>https://www.digikey.ca/en/products/detail/grayhill-inc/76SB08ST/726234</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/grayhill-inc/76SB08ST/726234</t>
+  </si>
+  <si>
+    <t>D9, D10, D12, D13, D14, D15, D16, D17, D18, D19, D20, D21</t>
   </si>
 </sst>
 </file>
@@ -1442,7 +1475,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F46"/>
+  <dimension ref="A1:F48"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.5" customWidth="1"/>
@@ -1729,6 +1762,23 @@
         <v>92</v>
       </c>
     </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A17">
+        <v>1</v>
+      </c>
+      <c r="B17" t="s">
+        <v>171</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="D17" t="s">
+        <v>173</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>174</v>
+      </c>
+    </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
         <v>59</v>
@@ -1736,10 +1786,10 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B20" t="s">
-        <v>171</v>
+        <v>182</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>28</v>
@@ -2070,43 +2120,80 @@
         <v>133</v>
       </c>
     </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A44">
+        <v>1</v>
+      </c>
+      <c r="B44" t="s">
+        <v>176</v>
+      </c>
+      <c r="C44" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D44" t="s">
+        <v>177</v>
+      </c>
+      <c r="F44" s="4" t="s">
+        <v>130</v>
+      </c>
+    </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A45">
-        <v>5</v>
-      </c>
-      <c r="B45" t="s">
-        <v>142</v>
-      </c>
-      <c r="C45" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="D45" s="13" t="s">
-        <v>134</v>
-      </c>
-      <c r="E45" s="14" t="s">
-        <v>138</v>
-      </c>
-      <c r="F45" s="4" t="s">
-        <v>135</v>
-      </c>
+      <c r="F45" s="4"/>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A46">
+        <v>1</v>
+      </c>
+      <c r="B46" t="s">
+        <v>178</v>
+      </c>
+      <c r="C46" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="D46" t="s">
+        <v>179</v>
+      </c>
+      <c r="F46" s="4" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A47">
+        <v>5</v>
+      </c>
+      <c r="B47" t="s">
+        <v>142</v>
+      </c>
+      <c r="C47" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="D47" s="13" t="s">
+        <v>134</v>
+      </c>
+      <c r="E47" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="F47" s="4" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A48">
         <v>2</v>
       </c>
-      <c r="B46" t="s">
+      <c r="B48" t="s">
         <v>141</v>
       </c>
-      <c r="C46" s="3" t="s">
+      <c r="C48" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="D46" s="13" t="s">
+      <c r="D48" s="13" t="s">
         <v>137</v>
       </c>
-      <c r="E46" s="14" t="s">
+      <c r="E48" s="14" t="s">
         <v>138</v>
       </c>
-      <c r="F46" s="4" t="s">
+      <c r="F48" s="4" t="s">
         <v>136</v>
       </c>
     </row>
@@ -2138,8 +2225,11 @@
     <hyperlink ref="F41" r:id="rId24" xr:uid="{DA5C4A80-C28F-614B-B024-A0121A23754C}"/>
     <hyperlink ref="F42" r:id="rId25" xr:uid="{0AEF5929-C21F-034C-9EF9-A59937EF5E30}"/>
     <hyperlink ref="F43" r:id="rId26" xr:uid="{A52DD678-1B51-054B-98C9-29F3B8135324}"/>
-    <hyperlink ref="F45" r:id="rId27" xr:uid="{587323B0-C77D-9E48-B2DC-DE4696097D1B}"/>
-    <hyperlink ref="F46" r:id="rId28" xr:uid="{5D66FE22-D23D-D44A-AD2B-E50B4B7816DF}"/>
+    <hyperlink ref="F47" r:id="rId27" xr:uid="{587323B0-C77D-9E48-B2DC-DE4696097D1B}"/>
+    <hyperlink ref="F48" r:id="rId28" xr:uid="{5D66FE22-D23D-D44A-AD2B-E50B4B7816DF}"/>
+    <hyperlink ref="F17" r:id="rId29" xr:uid="{DE9755CD-1102-284A-87EF-E52B7B77E18F}"/>
+    <hyperlink ref="F44" r:id="rId30" xr:uid="{6692828A-7FC3-9E44-9613-312074F3A70D}"/>
+    <hyperlink ref="F46" r:id="rId31" xr:uid="{8DCEA17E-5BF0-B749-A2E2-7B31BE802CDB}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2147,7 +2237,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3DC216C-48A1-2A43-8247-1510E9088A60}">
-  <dimension ref="A1:F46"/>
+  <dimension ref="A1:F48"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.5" customWidth="1"/>
@@ -2434,6 +2524,23 @@
         <v>92</v>
       </c>
     </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A17">
+        <v>1</v>
+      </c>
+      <c r="B17" t="s">
+        <v>171</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="D17" t="s">
+        <v>173</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>175</v>
+      </c>
+    </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
         <v>59</v>
@@ -2441,10 +2548,10 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B20" t="s">
-        <v>171</v>
+        <v>182</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>28</v>
@@ -2775,43 +2882,77 @@
         <v>168</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A45">
-        <v>5</v>
-      </c>
-      <c r="B45" t="s">
-        <v>142</v>
-      </c>
-      <c r="C45" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="D45" s="13" t="s">
-        <v>134</v>
-      </c>
-      <c r="E45" s="14" t="s">
-        <v>138</v>
-      </c>
-      <c r="F45" s="4" t="s">
-        <v>169</v>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A44">
+        <v>1</v>
+      </c>
+      <c r="B44" t="s">
+        <v>176</v>
+      </c>
+      <c r="C44" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D44" t="s">
+        <v>177</v>
+      </c>
+      <c r="F44" s="4" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A46">
+        <v>1</v>
+      </c>
+      <c r="B46" t="s">
+        <v>178</v>
+      </c>
+      <c r="C46" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="D46" t="s">
+        <v>179</v>
+      </c>
+      <c r="F46" s="4" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A47">
+        <v>5</v>
+      </c>
+      <c r="B47" t="s">
+        <v>142</v>
+      </c>
+      <c r="C47" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="D47" s="13" t="s">
+        <v>134</v>
+      </c>
+      <c r="E47" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="F47" s="4" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A48">
         <v>2</v>
       </c>
-      <c r="B46" t="s">
+      <c r="B48" t="s">
         <v>141</v>
       </c>
-      <c r="C46" s="3" t="s">
+      <c r="C48" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="D46" s="13" t="s">
+      <c r="D48" s="13" t="s">
         <v>137</v>
       </c>
-      <c r="E46" s="14" t="s">
+      <c r="E48" s="14" t="s">
         <v>138</v>
       </c>
-      <c r="F46" s="4" t="s">
+      <c r="F48" s="4" t="s">
         <v>170</v>
       </c>
     </row>
@@ -2843,8 +2984,11 @@
     <hyperlink ref="F41" r:id="rId24" xr:uid="{E5A12B65-D7C7-5A4C-8A60-DC956C69AF5F}"/>
     <hyperlink ref="F42" r:id="rId25" xr:uid="{C08F7662-C14D-EA47-812B-A25CCBF66167}"/>
     <hyperlink ref="F43" r:id="rId26" xr:uid="{4FB7BDC1-8001-DE45-9FD3-1AF429333A5F}"/>
-    <hyperlink ref="F45" r:id="rId27" xr:uid="{011F2CD8-F01A-EB48-B3E9-78ED4F91272D}"/>
-    <hyperlink ref="F46" r:id="rId28" xr:uid="{D795ACAA-CBE1-CB48-8DBF-705D816F14B1}"/>
+    <hyperlink ref="F47" r:id="rId27" xr:uid="{011F2CD8-F01A-EB48-B3E9-78ED4F91272D}"/>
+    <hyperlink ref="F48" r:id="rId28" xr:uid="{D795ACAA-CBE1-CB48-8DBF-705D816F14B1}"/>
+    <hyperlink ref="F17" r:id="rId29" xr:uid="{90EE06B8-80EB-2948-B611-E10B34708844}"/>
+    <hyperlink ref="F44" r:id="rId30" xr:uid="{84EB2F0D-B7E1-AC43-90F3-6BD8CEB7F198}"/>
+    <hyperlink ref="F46" r:id="rId31" xr:uid="{899FD64D-51FE-B84F-8A12-348633CBD36D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>